<commit_message>
auto: session 2026-08-20 10:03
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/Bao-Gia-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
+++ b/11-bao-gia-khach/Bao-Gia-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
@@ -2991,7 +2991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3075,17 +3075,15 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Phapluat.suckhoedoisong.vn</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>https://wiki.batdongsan.com.vn/</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>4940000</v>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>1 Link Dof</t>
+          <t>2 Link Nof</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -3093,11 +3091,7 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Mua thêm link 300k</t>
-        </is>
-      </c>
+      <c r="F8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -3105,15 +3099,15 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>https://wiki.batdongsan.com.vn/</t>
+          <t>thuonghieucongluan.com.vn</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>4940000</v>
+        <v>2185000</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>2 Link Nof</t>
+          <t>1000 từ 3 ảnh 1 link dof</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -3121,7 +3115,11 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Mua thêm link 400k</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -3129,15 +3127,15 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>thuonghieucongluan.com.vn</t>
+          <t>Suckhoephapluat.nguoiduatin.vn</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>2185000</v>
+        <v>1662000</v>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 1 link dof</t>
+          <t>2 Link Dofollow</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -3145,11 +3143,7 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Mua thêm link 400k</t>
-        </is>
-      </c>
+      <c r="F10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -3157,11 +3151,11 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Suckhoephapluat.nguoiduatin.vn</t>
+          <t>tuyensinhhuongnghiep.vn</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>1662000</v>
+        <v>1568000</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
@@ -3173,7 +3167,11 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>1000 từ 3 ảnh 2 link dof</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -3181,17 +3179,15 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Diendandoanhnghiep.vn</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>thanhnienviet.vn</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>1900000</v>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>2 Link Dofollow</t>
+          <t>2 link Dofollow</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -3201,7 +3197,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>700 từ + 3 ảnh</t>
+          <t>1500 từ 5 ảnh 2 link dof</t>
         </is>
       </c>
     </row>
@@ -3211,17 +3207,15 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Vietq.vn</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>Phunusuckhoe.giadinhonline.vn</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>1710000</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>2 Link Dofollow</t>
+          <t>1 link Doffollow</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -3229,7 +3223,11 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>1000 từ 3 ảnh 2 link dof</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
@@ -3237,27 +3235,25 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Nhipcaudautu.vn</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>thitruongngaynay.vn</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>665000</v>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>1 Link Dof(thêm link 500k)</t>
+          <t>2 Link Dofollow</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>SKDN</t>
+          <t>Mục phù hợp</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>300 từ 1 ảnh bài event</t>
+          <t>1000 từ 3 ảnh 2 link dof</t>
         </is>
       </c>
     </row>
@@ -3267,11 +3263,11 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>tuyensinhhuongnghiep.vn</t>
+          <t>suckhoegiadinhvietnam.com</t>
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>1568000</v>
+        <v>665000</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
@@ -3295,17 +3291,15 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Petrotimes.vn</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>Thuonghieuphattrien.com</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>665000</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>1 link Doffollow (thêm link 200k)</t>
+          <t>2 Link Dofollow</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -3313,7 +3307,11 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>1000 từ 3 ảnh 2 link dof</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -3321,13 +3319,11 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>nghean24h.vn</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>https://camnangsuckhoeso.net/</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>665000</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
@@ -3351,17 +3347,15 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Vnreview.vn</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>doisongphapluat.com.vn</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>1520000</v>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>2 link Dofollow</t>
+          <t>Không chèn link</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -3369,7 +3363,11 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>1000 từ  - 5 ảnh</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
@@ -3377,25 +3375,23 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Doanhnghiepvn.vn</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>Xaluannews.com</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>2090000</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>1 Link Dof(thêm link 300k)</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Bài đi lấy link</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr"/>
+          <t>1 link dof</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>1000 từ  - 3 ảnh - thêm link 500k/link</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
@@ -3403,27 +3399,21 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Nguoidothi.net.vn</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
+          <t>https://www.tinnhanhchungkhoan.vn/</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>3515000</v>
+      </c>
+      <c r="D20" s="8" t="inlineStr"/>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Loại 6 - Thông báo - Bố cáo</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>500 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 900 từ, 2 ảnh</t>
         </is>
       </c>
     </row>
@@ -3433,27 +3423,25 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Phunuvagiadinh.vn</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>https://vir.com.vn/</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>4664000</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>2 link Dofollow</t>
+          <t>Không gắn link</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Bài đi lấy link</t>
+          <t>Bài chuyên mục</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Dưới 1000 từ, 5 ảnh, không gắn link</t>
         </is>
       </c>
     </row>
@@ -3463,25 +3451,26 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>thanhnienviet.vn</t>
+          <t>https://2sao.vn//</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>1900000</v>
+        <v>2256000</v>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>2 link Dofollow</t>
+          <t>Thêm link: 6tr/link</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Top 12 trang chuyên mục trở xuống</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>1500 từ 5 ảnh 2 link dof</t>
+          <t>Bài PR dưới 1000 từ, 5 ảnh
+Thêm link: 6tr/link</t>
         </is>
       </c>
     </row>
@@ -3491,27 +3480,21 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Giadinhvaphapluat.vn</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
+          <t>https://nhipcaudautu.vn/</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>3658000</v>
+      </c>
+      <c r="D23" s="8" t="inlineStr"/>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>phapluatkinhdoanh</t>
+          <t>Tin ngắn 300 chữ</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Tin ngắn 300 chữ</t>
         </is>
       </c>
     </row>
@@ -3521,25 +3504,25 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Phunusuckhoe.giadinhonline.vn</t>
+          <t>https://reatimes.vn/</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>1710000</v>
+        <v>5263000</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>1 link Doffollow</t>
+          <t>Chỉ được gắn 1 link trong bài viết, thể hiện dưới dạng https:/.www,,,</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Loại 4 Chuyên mục</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Độ dài không quá 1,200 từ và 6 ảnh minh họa (Trừ bài phóng sự ảnh)</t>
         </is>
       </c>
     </row>
@@ -3549,27 +3532,21 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Doisongvietnam.vn</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
+          <t>https://theleader.vn/</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>5596000</v>
+      </c>
+      <c r="D25" s="8" t="inlineStr"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Nhịp cầu kinh doanh</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Bài viết có nội dung dưới 1,000 chữ và tối đa 3 ảnh minh họa</t>
         </is>
       </c>
     </row>
@@ -3579,27 +3556,21 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>suckhoeviet.org.vn</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
+          <t>https://bongdaplus.vn/</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>9405000</v>
+      </c>
+      <c r="D26" s="8" t="inlineStr"/>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Chuyên mục</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>1001 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 1000 từ, 5 ảnh</t>
         </is>
       </c>
     </row>
@@ -3609,19 +3580,13 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Vanhoavaphattrien.vn</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
+          <t>https://vietgiaitri.com/</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>2812000</v>
+      </c>
+      <c r="D27" s="8" t="inlineStr"/>
       <c r="E27" s="8" t="inlineStr">
         <is>
           <t>Mục phù hợp</t>
@@ -3629,7 +3594,7 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 1000 từ, 3 ảnh</t>
         </is>
       </c>
     </row>
@@ -3639,27 +3604,21 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Hoinhap.vanhoavaphattrien.vn</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
+          <t>https://www.otofun.net/</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>6128000</v>
+      </c>
+      <c r="D28" s="8" t="inlineStr"/>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Bài PR 4</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 800 từ, 3 ảnh</t>
         </is>
       </c>
     </row>
@@ -3669,27 +3628,26 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Golfviet.vn</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>https://www.bestie.vn/</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>2584000</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>2 Link Dofollow</t>
+          <t>Thêm link: 400K/link</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Tiểu mục</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 1000 từ, 5 - 8 ảnh
+Thêm link: 300K/link</t>
         </is>
       </c>
     </row>
@@ -3699,27 +3657,26 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Xahoi.com.vn</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>https://bongda24h.vn/</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>3468000</v>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>2 Link Dofollow</t>
+          <t>Thêm link: 550K/link</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Chuyên mục</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>1001 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 1000 từ, 5 ảnh
+Thêm link:500K/link</t>
         </is>
       </c>
     </row>
@@ -3729,27 +3686,21 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Daklak24h.com.vn</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>2 link Doffollow (thêm link 200k)</t>
-        </is>
-      </c>
+          <t>https://www.bongda.com.vn/</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>4370000</v>
+      </c>
+      <c r="D31" s="8" t="inlineStr"/>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Chuyên mục</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 1000 từ, 5 ảnh</t>
         </is>
       </c>
     </row>
@@ -3759,27 +3710,21 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Phunuhiendai.vn</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
+          <t>https://hoahoctro.tienphong.vn/</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>2527000</v>
+      </c>
+      <c r="D32" s="8" t="inlineStr"/>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Chuyên mục</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 800 từ, 4 ảnh</t>
         </is>
       </c>
     </row>
@@ -3789,27 +3734,21 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Suckhoecongdongonline.vn</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>1 link Dof(thêm link 500k)</t>
-        </is>
-      </c>
+          <t>2GAME.VN</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>2166000</v>
+      </c>
+      <c r="D33" s="8" t="inlineStr"/>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Tin thường</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
+          <t>Bài PR dưới 800 từ, 3 ảnh</t>
         </is>
       </c>
     </row>
@@ -3819,886 +3758,27 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Phapluatvacuocsong.vn</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
+          <t>https://tintuconline.com.vn/</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>2328000</v>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>2 Link Dofollow</t>
+          <t>Thêm link: 5tr/link</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Tiểu mục</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>1001 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="n">
-        <v>28</v>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Cafedautu.vn</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="n">
-        <v>29</v>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>Songdep.com.vn</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>Vnfinance.vn</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="n">
-        <v>31</v>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Bau.vn</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>2 link Doffollow</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>1001 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="n">
-        <v>32</v>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>khoahoccuocsong.com</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>2 link Dofollow</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F39" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="n">
-        <v>33</v>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>Hanghoathuonghieu.vn</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>2 link Doffollow</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="n">
-        <v>34</v>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>Home.vn</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>Tieudungtiepthi.vn</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F42" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n">
-        <v>36</v>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>kinhtethoidai.net</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>2 link Dofollow</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="n">
-        <v>37</v>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>thitruongngaynay.vn</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="n">
-        <v>665000</v>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>suckhoegiadinhvietnam.com</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="n">
-        <v>665000</v>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="n">
-        <v>39</v>
-      </c>
-      <c r="B46" s="8" t="inlineStr">
-        <is>
-          <t>Thuonghieuphattrien.com</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="n">
-        <v>665000</v>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>https://camnangsuckhoeso.net/</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="n">
-        <v>665000</v>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>2 Link Dofollow</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ 3 ảnh 2 link dof</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="n">
-        <v>41</v>
-      </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>doisongphapluat.com.vn</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="n">
-        <v>1520000</v>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Không chèn link</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ  - 5 ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="n">
-        <v>42</v>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>Xaluannews.com</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="n">
-        <v>2090000</v>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>1 link dof</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr"/>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>1000 từ  - 3 ảnh - thêm link 500k/link</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="n">
-        <v>43</v>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>https://www.tinnhanhchungkhoan.vn/</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="n">
-        <v>3515000</v>
-      </c>
-      <c r="D50" s="8" t="inlineStr"/>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Loại 6 - Thông báo - Bố cáo</t>
-        </is>
-      </c>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 900 từ, 2 ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="n">
-        <v>44</v>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>https://vir.com.vn/</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="n">
-        <v>4664000</v>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Không gắn link</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Bài chuyên mục</t>
-        </is>
-      </c>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>Dưới 1000 từ, 5 ảnh, không gắn link</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="B52" s="8" t="inlineStr">
-        <is>
-          <t>https://2sao.vn//</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="n">
-        <v>2256000</v>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Thêm link: 6tr/link</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Top 12 trang chuyên mục trở xuống</t>
-        </is>
-      </c>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 1000 từ, 5 ảnh
-Thêm link: 6tr/link</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="n">
-        <v>46</v>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>https://nhipcaudautu.vn/</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="n">
-        <v>3658000</v>
-      </c>
-      <c r="D53" s="8" t="inlineStr"/>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Tin ngắn 300 chữ</t>
-        </is>
-      </c>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>Tin ngắn 300 chữ</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="n">
-        <v>47</v>
-      </c>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>https://reatimes.vn/</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="n">
-        <v>5263000</v>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Chỉ được gắn 1 link trong bài viết, thể hiện dưới dạng https:/.www,,,</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Loại 4 Chuyên mục</t>
-        </is>
-      </c>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>Độ dài không quá 1,200 từ và 6 ảnh minh họa (Trừ bài phóng sự ảnh)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n">
-        <v>48</v>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>https://theleader.vn/</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="n">
-        <v>5596000</v>
-      </c>
-      <c r="D55" s="8" t="inlineStr"/>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Nhịp cầu kinh doanh</t>
-        </is>
-      </c>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>Bài viết có nội dung dưới 1,000 chữ và tối đa 3 ảnh minh họa</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="n">
-        <v>49</v>
-      </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>https://bongdaplus.vn/</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="n">
-        <v>9405000</v>
-      </c>
-      <c r="D56" s="8" t="inlineStr"/>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Chuyên mục</t>
-        </is>
-      </c>
-      <c r="F56" s="8" t="inlineStr">
-        <is>
           <t>Bài PR dưới 1000 từ, 5 ảnh</t>
         </is>
       </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>https://vietgiaitri.com/</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="n">
-        <v>2812000</v>
-      </c>
-      <c r="D57" s="8" t="inlineStr"/>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 1000 từ, 3 ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="n">
-        <v>51</v>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>https://www.otofun.net/</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="n">
-        <v>6128000</v>
-      </c>
-      <c r="D58" s="8" t="inlineStr"/>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR 4</t>
-        </is>
-      </c>
-      <c r="F58" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 800 từ, 3 ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="n">
-        <v>52</v>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>https://www.bestie.vn/</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="n">
-        <v>2584000</v>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Thêm link: 400K/link</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Tiểu mục</t>
-        </is>
-      </c>
-      <c r="F59" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 1000 từ, 5 - 8 ảnh
-Thêm link: 300K/link</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="n">
-        <v>53</v>
-      </c>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>https://bongda24h.vn/</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="n">
-        <v>3468000</v>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Thêm link: 550K/link</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Chuyên mục</t>
-        </is>
-      </c>
-      <c r="F60" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 1000 từ, 5 ảnh
-Thêm link:500K/link</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="n">
-        <v>54</v>
-      </c>
-      <c r="B61" s="8" t="inlineStr">
-        <is>
-          <t>https://www.bongda.com.vn/</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="n">
-        <v>4370000</v>
-      </c>
-      <c r="D61" s="8" t="inlineStr"/>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Chuyên mục</t>
-        </is>
-      </c>
-      <c r="F61" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 1000 từ, 5 ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="n">
-        <v>55</v>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>https://hoahoctro.tienphong.vn/</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="n">
-        <v>2527000</v>
-      </c>
-      <c r="D62" s="8" t="inlineStr"/>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Chuyên mục</t>
-        </is>
-      </c>
-      <c r="F62" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 800 từ, 4 ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="n">
-        <v>56</v>
-      </c>
-      <c r="B63" s="8" t="inlineStr">
-        <is>
-          <t>2GAME.VN</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="n">
-        <v>2166000</v>
-      </c>
-      <c r="D63" s="8" t="inlineStr"/>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Tin thường</t>
-        </is>
-      </c>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 800 từ, 3 ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="n">
-        <v>57</v>
-      </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>https://tintuconline.com.vn/</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="n">
-        <v>2328000</v>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Thêm link: 5tr/link</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Tiểu mục</t>
-        </is>
-      </c>
-      <c r="F64" s="8" t="inlineStr">
-        <is>
-          <t>Bài PR dưới 1000 từ, 5 ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="n">
-        <v>58</v>
-      </c>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>Hiện tại theo hợp đồng ký kết thì 100% là link dof, tuy nhiên có thể sau này các Báo thay đổi chính sách hoặc quy định của Nhà nước chuyển từ dof về nof thì mong quý khách hàng thông cảm.</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr"/>
-      <c r="E65" s="8" t="inlineStr"/>
-      <c r="F65" s="8" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="n">
-        <v>59</v>
-      </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>Khách hàng vui lòng check kỹ bài demo trước khi gửi, nếu sai sót do bạn thì báo không chỉnh sửa, chúng tôi cũng không chịu trách nhiệm. Bạn vẫn phải thanh toán đủ 100%.</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr"/>
-      <c r="E66" s="8" t="inlineStr"/>
-      <c r="F66" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4720,7 +3800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5415,230 +4495,6 @@
           <t>1500 từ  - 5 ảnh - 2 link dof</t>
         </is>
       </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n">
-        <v>36</v>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>KHÁCH HÀNG VUI LÒNG ĐỌC KỸ QUY ĐỊNH (CK MUA BÁO MẶC ĐỊNH ĐỒNG Ý)</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="n">
-        <v>37</v>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>Giá đã bao gồm content lên báo tỉnh, KH chỉ cần gửi anchor text và URL</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>Giá chưa bao gồm VAT 8%</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="n">
-        <v>39</v>
-      </c>
-      <c r="B46" s="8" t="inlineStr">
-        <is>
-          <t>Công ty có xuất hóa đơn VAT và hợp đồng đầy đủ cho KH công ty</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>Cọc tối thiểu 50% để viết bài và đăng báo, 100% với báo lớn</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="n">
-        <v>41</v>
-      </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>Chỉ nhận các bài viết lĩnh vực được cho phép của pháp luật.</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="n">
-        <v>42</v>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>Không quảng bá ngôn từ đả kích, tuyên truyền chống phá nhà nước, tác phẩm đồi trụy...</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="n">
-        <v>43</v>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>Cần có giấy phép kinh doanh đầy đủ.</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="n">
-        <v>44</v>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>Các đầu báo là sự quản lý của nhà nước - cục thông tin, nên khi bài viết đăng tải chúng tôi cam kết không bao giờ được xóa khi không có sự cho phép của KH nhưng còn link out ra ngoài thì báo có quyền xem gỡ bỏ nếu về sau trang đích của bạn chỉnh sửa vi phạm pháp luật hay tuyên truyền chống phá nhà nước, trang bị công an niêm phong....</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="B52" s="8" t="inlineStr">
-        <is>
-          <t>Bài đăng lên báo là tồn tại theo domain/chính sách từng báo. (BH tối thiểu 1 năm, TH site tạm dừng hoạt động, bất khả kháng không BH)</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="n">
-        <v>46</v>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>Hiện tại theo hợp đồng ký kết thì 100% chèn link dof và nof tùy theo từng site, tuy nhiên có thể sau này các Báo thay đổi chính sách hoặc quy định của Nhà nước chuyển từ dof về nof hoặc xóa bỏ không chèn link.</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="n">
-        <v>47</v>
-      </c>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>Khách hàng vui lòng check kỹ bài demo trước khi gửi, nếu sai sót do bạn thì báo không chỉnh sửa, chúng tôi cũng không chịu trách nhiệm. Bạn vẫn phải thanh toán đủ 100%.</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n">
-        <v>48</v>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Bài đăng là theo đúng chính sách báo/tin tức/tạp chí - nhưng có 1 số trường hợp trang báo do bị hack; làm sai pháp luật bị Nhà Nước xóa thì bài của KH trên đó cũng bị xóa hoặc mất, mong KH thông cảm và chấp nhận.</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="n">
-        <v>49</v>
-      </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>Khách hàng vui lòng đọc kỹ các quy định trên trước khi thanh toán, nếu không thắc mắc mặc định đồng ý với quy định của chúng tôi!</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>Liên hệ</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
auto: session 2026-08-20 10:07
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/Bao-Gia-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
+++ b/11-bao-gia-khach/Bao-Gia-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,50 @@
       <color rgb="000E8C7F"/>
     </font>
     <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="001C2035"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color theme="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="000563C1"/>
+      <sz val="12"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="000E8C7F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
@@ -70,6 +114,12 @@
     <font>
       <b val="1"/>
       <color rgb="00FF7A3D"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00FF7A3D"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -118,27 +168,25 @@
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -521,20 +569,26 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -542,6 +596,8 @@
           <t>MỤC LỤC - BẢNG GIÁ BOOKING BÁO &amp; PR</t>
         </is>
       </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -549,6 +605,13 @@
           <t>Kính gửi: Brand Kingsport</t>
         </is>
       </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -568,12 +631,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>PR Báo lớn</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="2" t="n">
         <v>77</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -583,12 +646,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Bài PR kèm Link Dofollow</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="2" t="n">
         <v>27</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -598,12 +661,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Báo tỉnh - địa phương</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="2" t="n">
         <v>35</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -613,12 +676,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Thông tin Digicom &amp; thanh toán</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -670,20 +733,38 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -691,6 +772,12 @@
           <t>PR BÁO LỚN</t>
         </is>
       </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -698,6 +785,21 @@
           <t>← Về Mục lục</t>
         </is>
       </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3008,20 +3110,35 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -3029,6 +3146,11 @@
           <t>BÀI PR KÈM LINK DOFOLLOW</t>
         </is>
       </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3036,6 +3158,19 @@
           <t>← Về Mục lục</t>
         </is>
       </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3815,20 +3950,29 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -3836,6 +3980,9 @@
           <t>BÁO TỈNH - ĐỊA PHƯƠNG</t>
         </is>
       </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3843,6 +3990,15 @@
           <t>← Về Mục lục</t>
         </is>
       </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -4529,6 +4685,11 @@
           <t>THÔNG TIN DIGICOM &amp; THANH TOÁN</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
@@ -4536,6 +4697,7 @@
           <t>1. Thông tin bên bán</t>
         </is>
       </c>
+      <c r="B3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -4609,12 +4771,17 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+    </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>2. Thông tin thanh toán</t>
         </is>
       </c>
+      <c r="B11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -4676,12 +4843,17 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+    </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
           <t>3. Phí soạn nội dung</t>
         </is>
       </c>
+      <c r="B18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -4707,12 +4879,17 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+    </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
           <t>4. Hiệu lực báo giá</t>
         </is>
       </c>
+      <c r="B22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">

</xml_diff>

<commit_message>
auto: session 2026-08-20 10:19
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/Bao-Gia-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
+++ b/11-bao-gia-khach/Bao-Gia-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
@@ -7,11 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Muc luc" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR bao lon" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link dof" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bao tinh" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thong tin &amp; Thanh toan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mục lục" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Báo lớn" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link Dofollow" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Báo tỉnh" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textlink Báo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textlink Home" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thông tin &amp; Thanh toán" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +100,15 @@
       <sz val="12"/>
     </font>
     <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <i val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="14"/>
     </font>
@@ -166,13 +177,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -181,12 +192,14 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -555,12 +568,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -678,15 +691,45 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Textlink Báo (gói sidebar)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Xem →</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Textlink Home</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Xem →</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Thông tin Digicom &amp; thanh toán</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Xem →</t>
         </is>
@@ -703,6 +746,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -718,13 +763,13 @@
   <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="132" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="69" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -852,10 +897,10 @@
           <t>PR loại 2 (Kinh doanh -  Thị trường tiêu dùng)</t>
         </is>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="11" t="n">
         <v>4275000</v>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -879,10 +924,10 @@
           <t>PR loại 2 (Thời trang Hitech/Công nghệ thông tin/Ô tô/Xe máy/Thể thao/Sức khỏe/Đẹp/Giải trí/Bạn trẻ cuộc sống/Ăn - Chơi/Giáo dục)</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="11" t="n">
         <v>3610000</v>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -906,10 +951,10 @@
           <t>PR loại 1 (2h trang chủ): Kinh doanh/Thị trường tiêu dùng/Thời trang Hitech/Công nghệ thông tin/Ô tô/Xe máy/Sức khỏe/Đẹp</t>
         </is>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="10" t="n">
         <v>9000000</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="11" t="n">
         <v>6935000</v>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -933,10 +978,10 @@
           <t>PR loại 1 (2h trang chủ): Thể thao/Giải trí/Bạn trẻ cuộc sống/Ăn - Chơi/Giáo dục</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="11" t="n">
         <v>4940000</v>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -964,10 +1009,10 @@
           <t>Tiểu mục Nhóm 2</t>
         </is>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="10" t="n">
         <v>13000000</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="11" t="n">
         <v>8740000</v>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -991,10 +1036,10 @@
           <t>Tiểu mục Nhóm 1</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="11" t="n">
         <v>9975000</v>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -1022,10 +1067,10 @@
           <t>Giáo dục, số hóa</t>
         </is>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="11" t="n">
         <v>8740000</v>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -1049,10 +1094,10 @@
           <t>Doanh nghiệp viết 1 - bài tồn tại 6 tháng</t>
         </is>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="11" t="n">
         <v>7410000</v>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -1076,10 +1121,10 @@
           <t>Doanh nghiệp viết 2 - bài  tồn tại 24 tháng</t>
         </is>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="11" t="n">
         <v>11210000</v>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -1103,10 +1148,10 @@
           <t>Doanh nghiệp viết 3 - bài  tồn tại theo domain</t>
         </is>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="11" t="n">
         <v>14535000</v>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -1134,10 +1179,10 @@
           <t>Trang chủ</t>
         </is>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="11" t="n">
         <v>7600000</v>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1161,10 +1206,10 @@
           <t>Chuyên mục</t>
         </is>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D19" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="11" t="n">
         <v>2755000</v>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1192,10 +1237,10 @@
           <t>Tiểu mục</t>
         </is>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="E20" s="10" t="n">
+      <c r="E20" s="11" t="n">
         <v>7030000</v>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1219,10 +1264,10 @@
           <t>Tiểu mục</t>
         </is>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="11" t="n">
         <v>8930000</v>
       </c>
       <c r="F21" s="8" t="inlineStr"/>
@@ -1242,10 +1287,10 @@
           <t>Chuyên mục</t>
         </is>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="11" t="n">
         <v>5225000</v>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1269,10 +1314,10 @@
           <t>Trang chủ</t>
         </is>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D23" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E23" s="11" t="n">
         <v>8170000</v>
       </c>
       <c r="F23" s="8" t="inlineStr"/>
@@ -1296,10 +1341,10 @@
           <t>Tiểu mục</t>
         </is>
       </c>
-      <c r="D24" s="8" t="n">
+      <c r="D24" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E24" s="11" t="n">
         <v>4180000</v>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1323,10 +1368,10 @@
           <t>Xem - Ăn - Chơi</t>
         </is>
       </c>
-      <c r="D25" s="8" t="n">
+      <c r="D25" s="10" t="n">
         <v>8000000</v>
       </c>
-      <c r="E25" s="10" t="n">
+      <c r="E25" s="11" t="n">
         <v>6270000</v>
       </c>
       <c r="F25" s="8" t="inlineStr"/>
@@ -1350,10 +1395,10 @@
           <t>PR cần biết</t>
         </is>
       </c>
-      <c r="D26" s="8" t="n">
+      <c r="D26" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="11" t="n">
         <v>3515000</v>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -1377,10 +1422,10 @@
           <t>Giáo dục, Du lịch, Giải trí, Giới trẻ, Văn hóa</t>
         </is>
       </c>
-      <c r="D27" s="8" t="n">
+      <c r="D27" s="10" t="n">
         <v>13000000</v>
       </c>
-      <c r="E27" s="10" t="n">
+      <c r="E27" s="11" t="n">
         <v>11381000</v>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -1404,10 +1449,10 @@
           <t>Kinh tế, Tiêu dùng, Công nghệ - Game, Đời sống, Sức khỏe, Thể thao, Emagazine, Xe</t>
         </is>
       </c>
-      <c r="D28" s="8" t="n">
+      <c r="D28" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="E28" s="10" t="n">
+      <c r="E28" s="11" t="n">
         <v>13252000</v>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -1435,10 +1480,10 @@
           <t>Chuyên Mục</t>
         </is>
       </c>
-      <c r="D29" s="8" t="n">
+      <c r="D29" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E29" s="10" t="n">
+      <c r="E29" s="11" t="n">
         <v>4275000</v>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -1462,10 +1507,10 @@
           <t>Bài thương hiệu</t>
         </is>
       </c>
-      <c r="D30" s="8" t="n">
+      <c r="D30" s="10" t="n">
         <v>9000000</v>
       </c>
-      <c r="E30" s="10" t="n">
+      <c r="E30" s="11" t="n">
         <v>6650000</v>
       </c>
       <c r="F30" s="8" t="inlineStr"/>
@@ -1485,10 +1530,10 @@
           <t>Trang chủ</t>
         </is>
       </c>
-      <c r="D31" s="8" t="n">
+      <c r="D31" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E31" s="11" t="n">
         <v>9975000</v>
       </c>
       <c r="F31" s="8" t="inlineStr"/>
@@ -1512,10 +1557,10 @@
           <t>Box Thông Cáo Báo chí (Trang chủ 1 ngày)</t>
         </is>
       </c>
-      <c r="D32" s="8" t="n">
+      <c r="D32" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E32" s="10" t="n">
+      <c r="E32" s="11" t="n">
         <v>5130000</v>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -1539,10 +1584,10 @@
           <t>Tin doanh nghiệp (Trang chủ 1 ngày)</t>
         </is>
       </c>
-      <c r="D33" s="8" t="n">
+      <c r="D33" s="10" t="n">
         <v>7500000</v>
       </c>
-      <c r="E33" s="10" t="n">
+      <c r="E33" s="11" t="n">
         <v>6270000</v>
       </c>
       <c r="F33" s="8" t="inlineStr"/>
@@ -1558,10 +1603,10 @@
           <t>Chuyên mục nhóm 2 (CM còn lại)</t>
         </is>
       </c>
-      <c r="D34" s="8" t="n">
+      <c r="D34" s="10" t="n">
         <v>8000000</v>
       </c>
-      <c r="E34" s="10" t="n">
+      <c r="E34" s="11" t="n">
         <v>6745000</v>
       </c>
       <c r="F34" s="8" t="inlineStr"/>
@@ -1581,10 +1626,10 @@
           <t>Chuyên mục 1 ((BDS, DN, Tài Chính - Ngân hàng, Chứng khoán. Smart Money)</t>
         </is>
       </c>
-      <c r="D35" s="8" t="n">
+      <c r="D35" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E35" s="10" t="n">
+      <c r="E35" s="11" t="n">
         <v>9880000</v>
       </c>
       <c r="F35" s="8" t="inlineStr"/>
@@ -1608,10 +1653,10 @@
           <t>Tin ngắn</t>
         </is>
       </c>
-      <c r="D36" s="8" t="n">
+      <c r="D36" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E36" s="10" t="n">
+      <c r="E36" s="11" t="n">
         <v>4560000</v>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -1635,10 +1680,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D37" s="8" t="n">
+      <c r="D37" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E37" s="10" t="n">
+      <c r="E37" s="11" t="n">
         <v>10260000</v>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -1666,10 +1711,10 @@
           <t>bài chuyên mục phù hợp</t>
         </is>
       </c>
-      <c r="D38" s="8" t="n">
+      <c r="D38" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E38" s="10" t="n">
+      <c r="E38" s="11" t="n">
         <v>4180000</v>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -1697,10 +1742,10 @@
           <t>Tiểu mục</t>
         </is>
       </c>
-      <c r="D39" s="8" t="n">
+      <c r="D39" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E39" s="10" t="n">
+      <c r="E39" s="11" t="n">
         <v>4750000</v>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -1728,10 +1773,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D40" s="8" t="n">
+      <c r="D40" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="E40" s="10" t="n">
+      <c r="E40" s="11" t="n">
         <v>2090000</v>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -1759,10 +1804,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D41" s="8" t="n">
+      <c r="D41" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="E41" s="10" t="n">
+      <c r="E41" s="11" t="n">
         <v>2090000</v>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -1790,10 +1835,10 @@
           <t>chuyên mục phù hợp</t>
         </is>
       </c>
-      <c r="D42" s="8" t="n">
+      <c r="D42" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E42" s="10" t="n">
+      <c r="E42" s="11" t="n">
         <v>3800000</v>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -1821,10 +1866,10 @@
           <t>Chuyên mục</t>
         </is>
       </c>
-      <c r="D43" s="8" t="n">
+      <c r="D43" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E43" s="10" t="n">
+      <c r="E43" s="11" t="n">
         <v>4180000</v>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -1852,10 +1897,10 @@
           <t>Chuyên mục</t>
         </is>
       </c>
-      <c r="D44" s="8" t="n">
+      <c r="D44" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E44" s="10" t="n">
+      <c r="E44" s="11" t="n">
         <v>4180000</v>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -1879,10 +1924,10 @@
           <t>Trang chủ steam 2</t>
         </is>
       </c>
-      <c r="D45" s="8" t="n">
+      <c r="D45" s="10" t="n">
         <v>8000000</v>
       </c>
-      <c r="E45" s="10" t="n">
+      <c r="E45" s="11" t="n">
         <v>6270000</v>
       </c>
       <c r="F45" s="8" t="inlineStr"/>
@@ -1906,10 +1951,10 @@
           <t>Mục doanh nghiệp - doanh nhân</t>
         </is>
       </c>
-      <c r="D46" s="8" t="n">
+      <c r="D46" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E46" s="10" t="n">
+      <c r="E46" s="11" t="n">
         <v>3230000</v>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -1933,10 +1978,10 @@
           <t>Trang tiểu mục</t>
         </is>
       </c>
-      <c r="D47" s="8" t="n">
+      <c r="D47" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E47" s="10" t="n">
+      <c r="E47" s="11" t="n">
         <v>3230000</v>
       </c>
       <c r="F47" s="8" t="inlineStr"/>
@@ -1956,10 +2001,10 @@
           <t>Trang chuyên mục</t>
         </is>
       </c>
-      <c r="D48" s="8" t="n">
+      <c r="D48" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E48" s="10" t="n">
+      <c r="E48" s="11" t="n">
         <v>3800000</v>
       </c>
       <c r="F48" s="8" t="inlineStr"/>
@@ -1983,10 +2028,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D49" s="8" t="n">
+      <c r="D49" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E49" s="10" t="n">
+      <c r="E49" s="11" t="n">
         <v>4275000</v>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -2014,10 +2059,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D50" s="8" t="n">
+      <c r="D50" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E50" s="10" t="n">
+      <c r="E50" s="11" t="n">
         <v>4275000</v>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -2045,10 +2090,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D51" s="8" t="n">
+      <c r="D51" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E51" s="10" t="n">
+      <c r="E51" s="11" t="n">
         <v>3420000</v>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -2076,10 +2121,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D52" s="8" t="n">
+      <c r="D52" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="E52" s="10" t="n">
+      <c r="E52" s="11" t="n">
         <v>1900000</v>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -2107,10 +2152,10 @@
           <t>Bài hot Tiểu mục</t>
         </is>
       </c>
-      <c r="D53" s="8" t="n">
+      <c r="D53" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E53" s="10" t="n">
+      <c r="E53" s="11" t="n">
         <v>3515000</v>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -2138,10 +2183,10 @@
           <t>Chuyên mục</t>
         </is>
       </c>
-      <c r="D54" s="8" t="n">
+      <c r="D54" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E54" s="10" t="n">
+      <c r="E54" s="11" t="n">
         <v>3610000</v>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -2169,10 +2214,10 @@
           <t>chuyên mục phù hợp</t>
         </is>
       </c>
-      <c r="D55" s="8" t="n">
+      <c r="D55" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="E55" s="10" t="n">
+      <c r="E55" s="11" t="n">
         <v>2755000</v>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -2200,10 +2245,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D56" s="8" t="n">
+      <c r="D56" s="10" t="n">
         <v>2000000</v>
       </c>
-      <c r="E56" s="10" t="n">
+      <c r="E56" s="11" t="n">
         <v>1520000</v>
       </c>
       <c r="F56" s="8" t="inlineStr">
@@ -2231,10 +2276,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D57" s="8" t="n">
+      <c r="D57" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E57" s="10" t="n">
+      <c r="E57" s="11" t="n">
         <v>8645000</v>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -2262,10 +2307,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D58" s="8" t="n">
+      <c r="D58" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="E58" s="10" t="n">
+      <c r="E58" s="11" t="n">
         <v>3040000</v>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -2293,10 +2338,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D59" s="8" t="n">
+      <c r="D59" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="E59" s="10" t="n">
+      <c r="E59" s="11" t="n">
         <v>4275000</v>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -2324,10 +2369,10 @@
           <t>Tin chuyên mục</t>
         </is>
       </c>
-      <c r="D60" s="8" t="n">
+      <c r="D60" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="E60" s="10" t="n">
+      <c r="E60" s="11" t="n">
         <v>3325000</v>
       </c>
       <c r="F60" s="8" t="inlineStr">
@@ -2355,10 +2400,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D61" s="8" t="n">
+      <c r="D61" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E61" s="10" t="n">
+      <c r="E61" s="11" t="n">
         <v>3800000</v>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -2386,10 +2431,10 @@
           <t>Bài loại 7 trang chuyên mục</t>
         </is>
       </c>
-      <c r="D62" s="8" t="n">
+      <c r="D62" s="10" t="n">
         <v>2000000</v>
       </c>
-      <c r="E62" s="10" t="n">
+      <c r="E62" s="11" t="n">
         <v>1900000</v>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -2417,10 +2462,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D63" s="8" t="n">
+      <c r="D63" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="E63" s="10" t="n">
+      <c r="E63" s="11" t="n">
         <v>5700000</v>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -2444,10 +2489,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D64" s="8" t="n">
+      <c r="D64" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="E64" s="10" t="n">
+      <c r="E64" s="11" t="n">
         <v>8550000</v>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -2471,10 +2516,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D65" s="8" t="n">
+      <c r="D65" s="10" t="n">
         <v>1500000</v>
       </c>
-      <c r="E65" s="10" t="n">
+      <c r="E65" s="11" t="n">
         <v>1330000</v>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -2502,10 +2547,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D66" s="8" t="n">
+      <c r="D66" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="E66" s="10" t="n">
+      <c r="E66" s="11" t="n">
         <v>3990000</v>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -2533,10 +2578,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D67" s="8" t="n">
+      <c r="D67" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="E67" s="10" t="n">
+      <c r="E67" s="11" t="n">
         <v>3230000</v>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -2564,10 +2609,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D68" s="8" t="n">
+      <c r="D68" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="E68" s="10" t="n">
+      <c r="E68" s="11" t="n">
         <v>2470000</v>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -2595,10 +2640,10 @@
           <t>Cần biết</t>
         </is>
       </c>
-      <c r="D69" s="8" t="n">
+      <c r="D69" s="10" t="n">
         <v>8000000</v>
       </c>
-      <c r="E69" s="10" t="n">
+      <c r="E69" s="11" t="n">
         <v>6175000</v>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -2626,10 +2671,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D70" s="8" t="n">
+      <c r="D70" s="10" t="n">
         <v>4800000</v>
       </c>
-      <c r="E70" s="10" t="n">
+      <c r="E70" s="11" t="n">
         <v>4275000</v>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -2657,10 +2702,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D71" s="8" t="n">
+      <c r="D71" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E71" s="10" t="n">
+      <c r="E71" s="11" t="n">
         <v>5130000</v>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -2688,10 +2733,10 @@
           <t>Chuyên mục</t>
         </is>
       </c>
-      <c r="D72" s="8" t="n">
+      <c r="D72" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E72" s="10" t="n">
+      <c r="E72" s="11" t="n">
         <v>5035000</v>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -2715,10 +2760,10 @@
           <t>Trang chủ</t>
         </is>
       </c>
-      <c r="D73" s="8" t="n">
+      <c r="D73" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E73" s="10" t="n">
+      <c r="E73" s="11" t="n">
         <v>8645000</v>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -2746,10 +2791,10 @@
           <t>Thông tin doanh nghiệp</t>
         </is>
       </c>
-      <c r="D74" s="8" t="n">
+      <c r="D74" s="10" t="n">
         <v>8000000</v>
       </c>
-      <c r="E74" s="10" t="n">
+      <c r="E74" s="11" t="n">
         <v>5700000</v>
       </c>
       <c r="F74" s="8" t="inlineStr">
@@ -2777,10 +2822,10 @@
           <t>Tin</t>
         </is>
       </c>
-      <c r="D75" s="8" t="n">
+      <c r="D75" s="10" t="n">
         <v>8000000</v>
       </c>
-      <c r="E75" s="10" t="n">
+      <c r="E75" s="11" t="n">
         <v>7125000</v>
       </c>
       <c r="F75" s="8" t="inlineStr">
@@ -2808,10 +2853,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D76" s="8" t="n">
+      <c r="D76" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E76" s="10" t="n">
+      <c r="E76" s="11" t="n">
         <v>5225000</v>
       </c>
       <c r="F76" s="8" t="inlineStr">
@@ -2839,10 +2884,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D77" s="8" t="n">
+      <c r="D77" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E77" s="10" t="n">
+      <c r="E77" s="11" t="n">
         <v>8360000</v>
       </c>
       <c r="F77" s="8" t="inlineStr">
@@ -2870,10 +2915,10 @@
           <t>TT doanh nghiệp</t>
         </is>
       </c>
-      <c r="D78" s="8" t="n">
+      <c r="D78" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="E78" s="10" t="n">
+      <c r="E78" s="11" t="n">
         <v>3705000</v>
       </c>
       <c r="F78" s="8" t="inlineStr">
@@ -2901,10 +2946,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D79" s="8" t="n">
+      <c r="D79" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="E79" s="10" t="n">
+      <c r="E79" s="11" t="n">
         <v>2660000</v>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -2932,10 +2977,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D80" s="8" t="n">
+      <c r="D80" s="10" t="n">
         <v>2000000</v>
       </c>
-      <c r="E80" s="10" t="n">
+      <c r="E80" s="11" t="n">
         <v>1615000</v>
       </c>
       <c r="F80" s="8" t="inlineStr">
@@ -2963,10 +3008,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D81" s="8" t="n">
+      <c r="D81" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="E81" s="10" t="n">
+      <c r="E81" s="11" t="n">
         <v>4750000</v>
       </c>
       <c r="F81" s="8" t="inlineStr">
@@ -2994,10 +3039,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D82" s="8" t="n">
+      <c r="D82" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="E82" s="10" t="n">
+      <c r="E82" s="11" t="n">
         <v>5890000</v>
       </c>
       <c r="F82" s="8" t="inlineStr">
@@ -3025,10 +3070,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D83" s="8" t="n">
+      <c r="D83" s="10" t="n">
         <v>3500000</v>
       </c>
-      <c r="E83" s="10" t="n">
+      <c r="E83" s="11" t="n">
         <v>2850000</v>
       </c>
       <c r="F83" s="8" t="inlineStr">
@@ -3056,10 +3101,10 @@
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D84" s="8" t="n">
+      <c r="D84" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="E84" s="10" t="n">
+      <c r="E84" s="11" t="n">
         <v>10355000</v>
       </c>
       <c r="F84" s="8" t="inlineStr">
@@ -3096,12 +3141,12 @@
   <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="69" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -3213,7 +3258,7 @@
           <t>https://wiki.batdongsan.com.vn/</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="10" t="n">
         <v>4940000</v>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -3237,7 +3282,7 @@
           <t>thuonghieucongluan.com.vn</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="10" t="n">
         <v>2185000</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -3265,7 +3310,7 @@
           <t>Suckhoephapluat.nguoiduatin.vn</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="10" t="n">
         <v>1662000</v>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -3289,7 +3334,7 @@
           <t>tuyensinhhuongnghiep.vn</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="10" t="n">
         <v>1568000</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -3317,7 +3362,7 @@
           <t>thanhnienviet.vn</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="10" t="n">
         <v>1900000</v>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -3345,7 +3390,7 @@
           <t>Phunusuckhoe.giadinhonline.vn</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="10" t="n">
         <v>1710000</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -3373,7 +3418,7 @@
           <t>thitruongngaynay.vn</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="10" t="n">
         <v>665000</v>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -3401,7 +3446,7 @@
           <t>suckhoegiadinhvietnam.com</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="10" t="n">
         <v>665000</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -3429,7 +3474,7 @@
           <t>Thuonghieuphattrien.com</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="10" t="n">
         <v>665000</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -3457,7 +3502,7 @@
           <t>https://camnangsuckhoeso.net/</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="10" t="n">
         <v>665000</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -3485,7 +3530,7 @@
           <t>doisongphapluat.com.vn</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="10" t="n">
         <v>1520000</v>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -3513,7 +3558,7 @@
           <t>Xaluannews.com</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="10" t="n">
         <v>2090000</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -3537,7 +3582,7 @@
           <t>https://www.tinnhanhchungkhoan.vn/</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="10" t="n">
         <v>3515000</v>
       </c>
       <c r="D20" s="8" t="inlineStr"/>
@@ -3561,7 +3606,7 @@
           <t>https://vir.com.vn/</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="10" t="n">
         <v>4664000</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -3589,7 +3634,7 @@
           <t>https://2sao.vn//</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22" s="10" t="n">
         <v>2256000</v>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -3618,7 +3663,7 @@
           <t>https://nhipcaudautu.vn/</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="10" t="n">
         <v>3658000</v>
       </c>
       <c r="D23" s="8" t="inlineStr"/>
@@ -3642,7 +3687,7 @@
           <t>https://reatimes.vn/</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
+      <c r="C24" s="10" t="n">
         <v>5263000</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -3670,7 +3715,7 @@
           <t>https://theleader.vn/</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n">
+      <c r="C25" s="10" t="n">
         <v>5596000</v>
       </c>
       <c r="D25" s="8" t="inlineStr"/>
@@ -3694,7 +3739,7 @@
           <t>https://bongdaplus.vn/</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C26" s="10" t="n">
         <v>9405000</v>
       </c>
       <c r="D26" s="8" t="inlineStr"/>
@@ -3718,7 +3763,7 @@
           <t>https://vietgiaitri.com/</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n">
+      <c r="C27" s="10" t="n">
         <v>2812000</v>
       </c>
       <c r="D27" s="8" t="inlineStr"/>
@@ -3742,7 +3787,7 @@
           <t>https://www.otofun.net/</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n">
+      <c r="C28" s="10" t="n">
         <v>6128000</v>
       </c>
       <c r="D28" s="8" t="inlineStr"/>
@@ -3766,7 +3811,7 @@
           <t>https://www.bestie.vn/</t>
         </is>
       </c>
-      <c r="C29" s="8" t="n">
+      <c r="C29" s="10" t="n">
         <v>2584000</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -3795,7 +3840,7 @@
           <t>https://bongda24h.vn/</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n">
+      <c r="C30" s="10" t="n">
         <v>3468000</v>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -3824,7 +3869,7 @@
           <t>https://www.bongda.com.vn/</t>
         </is>
       </c>
-      <c r="C31" s="8" t="n">
+      <c r="C31" s="10" t="n">
         <v>4370000</v>
       </c>
       <c r="D31" s="8" t="inlineStr"/>
@@ -3848,7 +3893,7 @@
           <t>https://hoahoctro.tienphong.vn/</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n">
+      <c r="C32" s="10" t="n">
         <v>2527000</v>
       </c>
       <c r="D32" s="8" t="inlineStr"/>
@@ -3872,7 +3917,7 @@
           <t>2GAME.VN</t>
         </is>
       </c>
-      <c r="C33" s="8" t="n">
+      <c r="C33" s="10" t="n">
         <v>2166000</v>
       </c>
       <c r="D33" s="8" t="inlineStr"/>
@@ -3896,7 +3941,7 @@
           <t>https://tintuconline.com.vn/</t>
         </is>
       </c>
-      <c r="C34" s="8" t="n">
+      <c r="C34" s="10" t="n">
         <v>2328000</v>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -3938,10 +3983,10 @@
   <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="69" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -4031,7 +4076,7 @@
           <t>Angiangtv.vn</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="10" t="n">
         <v>846000</v>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -4049,7 +4094,7 @@
           <t>Baodanang.vn</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="10" t="n">
         <v>950000</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -4067,7 +4112,7 @@
           <t>Baotuyenquang.com.vn</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="10" t="n">
         <v>998000</v>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -4085,7 +4130,7 @@
           <t>Baothanhhoa.vn</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="10" t="n">
         <v>1425000</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -4103,7 +4148,7 @@
           <t>Baohatinh.vn</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="10" t="n">
         <v>998000</v>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -4121,7 +4166,7 @@
           <t>baodongnai.com.vn</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="10" t="n">
         <v>1045000</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -4139,7 +4184,7 @@
           <t>Baoangiang.com.vn</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="10" t="n">
         <v>1140000</v>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -4157,7 +4202,7 @@
           <t>Baothainguyen.vn</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="10" t="n">
         <v>1425000</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -4175,7 +4220,7 @@
           <t>https://phunumoi.net.vn/</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="10" t="n">
         <v>1140000</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -4193,7 +4238,7 @@
           <t>baolamdong.vn</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="10" t="n">
         <v>1520000</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -4211,7 +4256,7 @@
           <t>Baotayninh.vn</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="10" t="n">
         <v>1472000</v>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -4229,7 +4274,7 @@
           <t>Sohuutritue.net.vn</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="10" t="n">
         <v>1472000</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -4247,7 +4292,7 @@
           <t>Baocantho.com.vn</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="10" t="n">
         <v>1520000</v>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -4265,7 +4310,7 @@
           <t>Baoquangninh.vn</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="10" t="n">
         <v>1520000</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -4283,7 +4328,7 @@
           <t>baodienbienphu.vn</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22" s="10" t="n">
         <v>1140000</v>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -4301,7 +4346,7 @@
           <t>baophutho.vn</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="10" t="n">
         <v>1235000</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -4319,7 +4364,7 @@
           <t>baolangson.vn</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
+      <c r="C24" s="10" t="n">
         <v>1710000</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -4337,7 +4382,7 @@
           <t>baocamau.vn</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n">
+      <c r="C25" s="10" t="n">
         <v>1330000</v>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -4355,7 +4400,7 @@
           <t>baovinhlong.com.vn</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C26" s="10" t="n">
         <v>1282000</v>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -4373,7 +4418,7 @@
           <t>baodongthap.vn</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n">
+      <c r="C27" s="10" t="n">
         <v>2755000</v>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -4391,7 +4436,7 @@
           <t>https://vietstock.vn/</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n">
+      <c r="C28" s="10" t="n">
         <v>1899000</v>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -4409,7 +4454,7 @@
           <t>baoquangtri.vn (mới về)</t>
         </is>
       </c>
-      <c r="C29" s="8" t="n">
+      <c r="C29" s="10" t="n">
         <v>1710000</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -4427,7 +4472,7 @@
           <t>Baocaobang.vn</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n">
+      <c r="C30" s="10" t="n">
         <v>1710000</v>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -4445,7 +4490,7 @@
           <t>https://baolaocai.vn/</t>
         </is>
       </c>
-      <c r="C31" s="8" t="n">
+      <c r="C31" s="10" t="n">
         <v>3610000</v>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -4463,7 +4508,7 @@
           <t>baodaklak.vn</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n">
+      <c r="C32" s="10" t="n">
         <v>4275000</v>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -4481,7 +4526,7 @@
           <t>baoxaydung.vn</t>
         </is>
       </c>
-      <c r="C33" s="8" t="n">
+      <c r="C33" s="10" t="n">
         <v>1805000</v>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -4499,7 +4544,7 @@
           <t>tapchixaydung.vn</t>
         </is>
       </c>
-      <c r="C34" s="8" t="n">
+      <c r="C34" s="10" t="n">
         <v>1995000</v>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -4517,7 +4562,7 @@
           <t>Vietbao.vn</t>
         </is>
       </c>
-      <c r="C35" s="8" t="n">
+      <c r="C35" s="10" t="n">
         <v>1881000</v>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -4535,7 +4580,7 @@
           <t>Thethaovanhoa.vn</t>
         </is>
       </c>
-      <c r="C36" s="8" t="n">
+      <c r="C36" s="10" t="n">
         <v>1900000</v>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -4553,7 +4598,7 @@
           <t>Bienphong.com.vn</t>
         </is>
       </c>
-      <c r="C37" s="8" t="n">
+      <c r="C37" s="10" t="n">
         <v>1330000</v>
       </c>
       <c r="D37" s="8" t="inlineStr">
@@ -4571,7 +4616,7 @@
           <t>anninhthudo.vn</t>
         </is>
       </c>
-      <c r="C38" s="8" t="n">
+      <c r="C38" s="10" t="n">
         <v>2470000</v>
       </c>
       <c r="D38" s="8" t="inlineStr">
@@ -4589,7 +4634,7 @@
           <t>thuonghieuvaphapluat.vn</t>
         </is>
       </c>
-      <c r="C39" s="8" t="n">
+      <c r="C39" s="10" t="n">
         <v>1615000</v>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -4607,7 +4652,7 @@
           <t>kinhtemoitruong.vn</t>
         </is>
       </c>
-      <c r="C40" s="8" t="n">
+      <c r="C40" s="10" t="n">
         <v>2850000</v>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -4625,7 +4670,7 @@
           <t>http://giaoducthudo.giaoducthoidai.vn/</t>
         </is>
       </c>
-      <c r="C41" s="8" t="n">
+      <c r="C41" s="10" t="n">
         <v>1425000</v>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -4643,7 +4688,7 @@
           <t>nguoihanoi.vn</t>
         </is>
       </c>
-      <c r="C42" s="8" t="n">
+      <c r="C42" s="10" t="n">
         <v>2280000</v>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -4672,11 +4717,2526 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="101" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TEXTLINK BÁO - GÓI SIDEBAR BÀI VIẾT</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>← Về Mục lục</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Gói textlink đặt đồng loạt trên nhiều trang báo (không chọn riêng từng báo). Đơn hàng từ 2 gói trở lên được hỗ trợ chiết khấu thêm - liên hệ để biết chi tiết.</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Gói</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Giá niêm yết</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Giá ưu đãi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Gói A1</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar bài viết 3 tháng</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1000 link sidebar bài viết Tặng 200 link free Đặt trên 30-37 trang báo Giới hạn 35 từ khoá</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>1758000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Gói A2</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar bài viết 3 tháng</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1500 link sidebar bài viết Tặng 200 link free Đặt trên 30-37 trang báo Giới hạn 40 từ khoá</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>2565000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Gói A3</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar bài viết 3 tháng</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>2000 link sidebar bài viết Tặng 200 link free Đặt trên 30-37 trang báo Giới hạn 50 từ khoá</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>3900000</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>3420000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Gói A4</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar bài viết 3 tháng</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>3000 link sidebar bài viết Tặng 200 link free Đặt trên 30-37 trang báo Giới hạn 50 từ khoá</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>5600000</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Gói A5</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar bài viết 3 tháng</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>5000 link sidebar bài viết Tặng 200 link free Đặt trên 30-37 trang báo Giới hạn 80 từ khoá</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>8800000</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>6840000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Gói A6</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar bài viết 3 tháng</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>10000 link sidebar bài viết Tặng 200 link free Đặt trên 30-37 trang báo Giới hạn 100 từ khoá</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>16800000</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>13300000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Gói A7</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar bài viết 3 tháng</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>15000 link sidebar bài viết Tặng 200 link free Đặt trên 30-37 trang báo Giới hạn 120 từ khoá</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>24000000</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>21850000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Gói B2</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Gói B (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1500 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 50 từ khoá</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>5100000</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>3800000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Gói B3</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Gói B (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>2000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 50 từ khoá</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>6400000</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>5130000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Gói B4</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Gói B (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>3000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 50 từ khoá</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>7078000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Gói B5</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Gói B (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>5000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 80 từ khoá</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>14800000</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>11400000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Gói B6</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Gói B (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>10000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 100 từ khoá</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>26800000</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>20900000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Gói B7</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Gói B (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>15000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 120 từ khoá</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>33250000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Gói C2</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Gói C (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1500 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 50 từ khoá</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>5510000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Gói C3</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Gói C (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>2000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 50 từ khoá</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>9700000</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>7410000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Gói C4</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Gói C (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>3000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 50 từ khoá</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="F24" s="11" t="n">
+        <v>11115000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Gói C5</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Gói C (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>5000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 80 từ khoá</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="F25" s="11" t="n">
+        <v>17432000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Gói C6</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Gói C (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>10000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 100 từ khoá</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>43800000</v>
+      </c>
+      <c r="F26" s="11" t="n">
+        <v>34865000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Gói C7</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Gói C (mở rộng)</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>15000 link sidebar bài viết - Tặng 200 link free - Đặt trên 30-37 trang báo - Giới hạn 120 từ khoá</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>62800000</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>50112000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Áp dụng trên 33 trang báo (danh sách minh hoạ, có thể thay đổi theo đợt triển khai):</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>hanoitimes.vn, thieunien.vn, thanhnienviet.vn, tapchinghiencuuphathoc.vn, www.phunuvagiadinh.vn, reatimes.vn, doanhnghiephoinhap.vn, baothainguyen.vn, huengaynay.vn, baocamau.vn, baotuyenquang.com.vn, baogialai.com.vn, nguoidothi.net.vn, baolangson.vn, baolaocai.vn, baoangiang.com.vn, baocantho.com.vn, truyenhinhnghean.vn, thuonghieucongluan.com.vn, baovanhoa.vn, tapchitoaan.vn, baodanang.vn, baodongnai.com.vn, giaoducthoidai.vn, baophapluat.vn, vnreview.vn, home.vn, congly.vn, www.anninhthudo.vn, hanoimoi.vn, thuonghieuvaphapluat.vn, anhp.vn, vietq.vn</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A29:F29"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000E8C7F"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="57" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TEXTLINK HOME</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>← Về Mục lục</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Giá theo 3 mức thời hạn: 3 tháng / 6 tháng / 12 tháng.</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Đơn vị</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Traffic/tháng</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>DR</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Giá Link Home</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Giá Link Chuyên mục</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Giá Link Fullsite</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="n"/>
+      <c r="N8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>3 tháng</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>6 tháng</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>12 tháng</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>3 tháng</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>6 tháng</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>12 tháng</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>3 tháng</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>6 tháng</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>12 tháng</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>hanoitimes.vn</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Báo điện tử Pháp luật và xã hội</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>101.000</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>1045000</v>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L10" s="10" t="n">
+        <v>950000</v>
+      </c>
+      <c r="M10" s="10" t="n">
+        <v>1140000</v>
+      </c>
+      <c r="N10" s="10" t="n">
+        <v>1330000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>thieunien.vn</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Trung ương Đoàn TNCS Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>56.000</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>1045000</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>950000</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>1140000</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>1330000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>thanhnienviet.vn</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Tạp chí điện tử thanhnienviet.vn</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>52.000</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>1045000</v>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K12" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L12" s="10" t="n">
+        <v>950000</v>
+      </c>
+      <c r="M12" s="10" t="n">
+        <v>1140000</v>
+      </c>
+      <c r="N12" s="10" t="n">
+        <v>1330000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>tapchinghiencuuphathoc.vn</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Tạp chí nghiên cứu Phật học</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>78.000</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>1045000</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K13" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L13" s="10" t="n">
+        <v>950000</v>
+      </c>
+      <c r="M13" s="10" t="n">
+        <v>1140000</v>
+      </c>
+      <c r="N13" s="10" t="n">
+        <v>1330000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>www.phunuvagiadinh.vn</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>TẠP CHÍ ĐIỆN TỬ PHỤ NỮ VÀ GIA ĐÌNH</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>135.000</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>1045000</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K14" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L14" s="10" t="n">
+        <v>950000</v>
+      </c>
+      <c r="M14" s="10" t="n">
+        <v>1140000</v>
+      </c>
+      <c r="N14" s="10" t="n">
+        <v>1330000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>reatimes.vn</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Hiệp hội Bất động sản Việt Nam (VNREA)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>89.000</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>1045000</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K15" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L15" s="10" t="n">
+        <v>950000</v>
+      </c>
+      <c r="M15" s="10" t="n">
+        <v>1140000</v>
+      </c>
+      <c r="N15" s="10" t="n">
+        <v>1330000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>doanhnghiephoinhap.vn</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>TẠP CHÍ ĐIỆN TỬ DOANH NGHIỆP VÀ HỘI NHẬP</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>880.000</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K16" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L16" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M16" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N16" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>baothainguyen.vn</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Thái Nguyên</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>400.000</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K17" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L17" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M17" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N17" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>huengaynay.vn</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN Tỉnh Thừa Thiên Huế</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>300.000</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K18" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L18" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M18" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N18" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>baocamau.vn</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Cà Mau</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>150.000</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K19" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L19" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M19" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N19" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>baotuyenquang.com.vn</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Tuyên Quang</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>270.000</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K20" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L20" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M20" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N20" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>baogialai.com.vn</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Gia Lai</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>210.000</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I21" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J21" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K21" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L21" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M21" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N21" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>nguoidothi.net.vn</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Tạp chí điện tử Người Đô Thị</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>322.000</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I22" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J22" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K22" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L22" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M22" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N22" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>baolangson.vn</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Lạng Sơn</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>350.000</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I23" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J23" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K23" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M23" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N23" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>baolaocai.vn</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Lào Cai</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>290.000</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H24" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I24" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J24" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K24" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L24" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M24" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N24" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>baoangiang.com.vn</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh An Giang</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>780.000</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G25" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I25" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K25" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L25" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M25" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N25" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>baocantho.com.vn</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Cần Thơ</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1.300.000</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H26" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I26" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J26" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K26" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L26" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M26" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N26" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>truyenhinhnghean.vn</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Đài phát thanh truyền hình Nghệ An</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>470.000</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I27" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K27" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L27" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M27" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N27" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>thuonghieucongluan.com.vn</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Tạp chí điện tử Thương hiệu và Công luận</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>365.000</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H28" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I28" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K28" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L28" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M28" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N28" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>baovanhoa.vn</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Báo điện tử Báo Văn Hoá</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>597.000</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H29" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I29" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J29" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K29" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L29" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M29" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N29" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>tapchitoaan.vn</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Tạp chí điện tử Toà án nhân dân</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>339.000</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="H30" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="I30" s="10" t="n">
+        <v>475000</v>
+      </c>
+      <c r="J30" s="10" t="n">
+        <v>570000</v>
+      </c>
+      <c r="K30" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="L30" s="10" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="M30" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="N30" s="10" t="n">
+        <v>4275000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>baodanang.vn</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>2.330.000</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H31" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I31" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J31" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K31" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L31" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M31" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N31" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>baodongnai.com.vn</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của đảng bộ ĐCS VN tỉnh Đồng Nai</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1.600.000</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H32" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I32" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J32" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K32" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L32" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M32" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N32" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>giaoducthoidai.vn</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan của Bộ Kế hoạch</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>7.000.000</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G33" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H33" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I33" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K33" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L33" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M33" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N33" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>baophapluat.vn</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Báo điện tử Pháp luật Việt Nam</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>2.600.000</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H34" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I34" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J34" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K34" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L34" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M34" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N34" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>vnreview.vn</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH VIỆT NAM ĐÁNH GIÁ</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1.400.000</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G35" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H35" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I35" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J35" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K35" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L35" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M35" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N35" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>home.vn</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH VIỆT NAM ĐÁNH GIÁ</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>2.200.000</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H36" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I36" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J36" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K36" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L36" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M36" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N36" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>congly.vn</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan ngôn luận toà án nhân dân tối cao</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>2.300.000</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H37" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I37" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J37" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K37" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L37" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M37" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N37" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>www.anninhthudo.vn</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan công an thành phố Hà Nội</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>4.000.000</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H38" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I38" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J38" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K38" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L38" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M38" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N38" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>hanoimoi.vn</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Báo điện tử Hà Nội Mới</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>2.100.000</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>2850000</v>
+      </c>
+      <c r="G39" s="10" t="n">
+        <v>3325000</v>
+      </c>
+      <c r="H39" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="I39" s="10" t="n">
+        <v>665000</v>
+      </c>
+      <c r="J39" s="10" t="n">
+        <v>760000</v>
+      </c>
+      <c r="K39" s="10" t="n">
+        <v>855000</v>
+      </c>
+      <c r="L39" s="10" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="M39" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="N39" s="10" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000E8C7F"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="140" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4692,7 +7252,7 @@
       <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>1. Thông tin bên bán</t>
         </is>
@@ -4705,7 +7265,7 @@
           <t>Tên công ty</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
@@ -4717,7 +7277,7 @@
           <t>Mã số thuế</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>0109816406</t>
         </is>
@@ -4729,7 +7289,7 @@
           <t>Địa chỉ giao dịch</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Số nhà 200, Đường 3.1, Khu đô thị Gamuda Garden, Phường Trần Phú, Quận Hoàng Mai, TP. Hà Nội</t>
         </is>
@@ -4741,7 +7301,7 @@
           <t>Hotline</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>0988 769 317</t>
         </is>
@@ -4753,7 +7313,7 @@
           <t>Email</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>sales@digicomvn.com</t>
         </is>
@@ -4765,7 +7325,7 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>digicomvn.com</t>
         </is>
@@ -4776,7 +7336,7 @@
       <c r="B10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>2. Thông tin thanh toán</t>
         </is>
@@ -4789,7 +7349,7 @@
           <t>Số tài khoản</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>567898838</t>
         </is>
@@ -4801,7 +7361,7 @@
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Ngân hàng TMCP Quân đội (MB Bank)</t>
         </is>
@@ -4813,7 +7373,7 @@
           <t>Chủ tài khoản</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
@@ -4825,7 +7385,7 @@
           <t>Nội dung chuyển khoản</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>[Số báo giá/mã đơn] + [Họ tên người chuyển]</t>
         </is>
@@ -4837,7 +7397,7 @@
           <t>Hình thức thanh toán</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Thanh toán 100% giá trị đơn hàng trước khi triển khai đăng bài. Đơn giá trị lớn/khách mới có thể áp dụng đặt cọc 50% - liên hệ để thống nhất trước khi đặt.</t>
         </is>
@@ -4848,7 +7408,7 @@
       <c r="B17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>3. Phí soạn nội dung</t>
         </is>
@@ -4861,7 +7421,7 @@
           <t>Viết bài PR</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>MIỄN PHÍ 100% - Digicom biên tập bài PR từ tư liệu khách cung cấp, không thu thêm phí.</t>
         </is>
@@ -4873,7 +7433,7 @@
           <t>Phụ phí (nếu có)</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Chỉ phát sinh 1.000.000đ/buổi nếu khách yêu cầu cử phóng viên đến tận nơi tác nghiệp (thay vì Digicom biên tập từ tư liệu khách gửi).</t>
         </is>
@@ -4884,7 +7444,7 @@
       <c r="B21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>4. Hiệu lực báo giá</t>
         </is>
@@ -4897,7 +7457,7 @@
           <t>Ngày phát hành</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>20/08/2026</t>
         </is>
@@ -4909,7 +7469,7 @@
           <t>Hiệu lực đến hết</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>27/08/2026 (7 ngày kể từ ngày phát hành)</t>
         </is>
@@ -4921,7 +7481,7 @@
           <t>Lưu ý</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Sau thời hạn trên, giá có thể thay đổi theo chính sách nhà cung cấp - vui lòng liên hệ để xác nhận lại giá trước khi đặt.</t>
         </is>

</xml_diff>

<commit_message>
auto: session 2026-08-20 10:21
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/Bao-Gia-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
+++ b/11-bao-gia-khach/Bao-Gia-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
@@ -180,7 +180,7 @@
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -585,7 +585,7 @@
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="46" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
@@ -594,7 +594,7 @@
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="46" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
@@ -785,7 +785,7 @@
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
@@ -798,7 +798,7 @@
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
@@ -3161,7 +3161,7 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
@@ -3173,7 +3173,7 @@
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
@@ -3999,7 +3999,7 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="46" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
@@ -4009,7 +4009,7 @@
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="46" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
@@ -4740,7 +4740,7 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
@@ -4752,7 +4752,7 @@
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
@@ -5428,7 +5428,7 @@
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
@@ -5448,7 +5448,7 @@
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>

</xml_diff>